<commit_message>
Update patent review for slope model and AimPoint
</commit_message>
<xml_diff>
--- a/docs/competitive_patent/PuttPhysics_競合・特許チェック表_Ver1.xlsx
+++ b/docs/competitive_patent/PuttPhysics_競合・特許チェック表_Ver1.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="競合チェック" sheetId="1" r:id="R73600b1cdf5f49c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PuttPhysics機能台帳" sheetId="2" r:id="R7a9a579ec0cd4fab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="特許深掘り" sheetId="3" r:id="R9d151d43c20149d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="4" r:id="Ra8ceefacbc91457d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="競合チェック" sheetId="1" r:id="R77ba4db5aaa54e12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PuttPhysics機能台帳" sheetId="2" r:id="R1748f243c0474d66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="特許深掘り" sheetId="3" r:id="R2dad00a57986404a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="4" r:id="R1635d2fa87984e57"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,7 +79,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="49">
+  <x:cellXfs count="51">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -182,6 +182,10 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -193,14 +197,14 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -210,14 +214,14 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -869,6 +873,53 @@
         <x:v>Ver.1で新たに監視対象へ追加</x:v>
       </x:c>
     </x:row>
+    <x:row r="9" ht="78" customHeight="1">
+      <x:c r="A9" s="12" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" s="12" t="str">
+        <x:v>AimPoint関連 / Putting Guide</x:v>
+      </x:c>
+      <x:c r="C9" s="12" t="str">
+        <x:v>傾斜・距離・グリーンスピード等からブレーク量/aim point/開始速度を扱うパッティング支援</x:v>
+      </x:c>
+      <x:c r="D9" s="12" t="str">
+        <x:v>グリーン傾斜・距離・速度情報＋参照ガイド/コンピュータ処理。下り方向を基準に時計文字盤で角度表現する記載あり</x:v>
+      </x:c>
+      <x:c r="E9" s="12" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="F9" s="12" t="str">
+        <x:v>将来：時計文字盤＋傾斜量、局所傾斜の逐次軌道計算、狙い方向/必要速度</x:v>
+      </x:c>
+      <x:c r="G9" s="12" t="str">
+        <x:v>傾斜・距離・グリーンスピード・ブレーク/狙い方向を扱う点</x:v>
+      </x:c>
+      <x:c r="H9" s="12" t="str">
+        <x:v>PuttPhysicsは各地点の局所傾斜とボール状態を逐次更新する物理シミュレーションを候補としており、静的参照ガイド等とは異なる可能性。ただし請求項比較が必要</x:v>
+      </x:c>
+      <x:c r="I9" s="12" t="str">
+        <x:v>US 7,988,572 B1 / US 8,162,779 B1 / US 2013/0116067 A1（関連ファミリー等を要確認）</x:v>
+      </x:c>
+      <x:c r="J9" s="12" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="K9" s="12" t="str">
+        <x:v>重点調査追加</x:v>
+      </x:c>
+      <x:c r="L9" s="12" t="str">
+        <x:v>時計文字盤・傾斜・距離・グリーンスピード・break/aim point/starting velocityの各要素を独立請求項と対応付け。対象国・法的状態・関連ファミリーも確認</x:v>
+      </x:c>
+      <x:c r="M9" s="12" t="str">
+        <x:v>2026-08-17</x:v>
+      </x:c>
+      <x:c r="N9" s="12" t="str">
+        <x:v>https://patents.google.com/patent/US8162779B1/en</x:v>
+      </x:c>
+      <x:c r="O9" s="12" t="str">
+        <x:v>現時点で非侵害判断はしない。US8162779B1/US7988572B1はGoogle Patents上でExpired - Fee Related表示だが、関連権利・各国・他特許は別途確認</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="J2:J8">
     <x:cfRule type="expression" dxfId="0" priority="1">
@@ -885,7 +936,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24051525759043ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf60452e69f9845d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1252,6 +1303,84 @@
         <x:v>競合差別化と知財の両面で重要</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="58" customHeight="1">
+      <x:c r="A15" s="12" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="str">
+        <x:v>局所傾斜による軌道計算</x:v>
+      </x:c>
+      <x:c r="C15" s="12" t="str">
+        <x:v>検討中</x:v>
+      </x:c>
+      <x:c r="D15" s="12" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E15" s="12" t="str">
+        <x:v>現在位置・速度・進行方向・回転状態と各地点の局所傾斜を逐次適用する物理モデルを検討</x:v>
+      </x:c>
+      <x:c r="F15" s="12" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="G15" s="12" t="str">
+        <x:v>物理モデル実装前</x:v>
+      </x:c>
+      <x:c r="H15" s="12" t="str">
+        <x:v>一定傾斜・複合傾斜・スネークラインを同じ基本モデルで扱う構想。AimPoint関連特許を要確認</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="58" customHeight="1">
+      <x:c r="A16" s="12" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B16" s="12" t="str">
+        <x:v>時計文字盤＋傾斜量入力</x:v>
+      </x:c>
+      <x:c r="C16" s="12" t="str">
+        <x:v>検討中</x:v>
+      </x:c>
+      <x:c r="D16" s="12" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E16" s="12" t="str">
+        <x:v>傾斜方向を時計文字盤、傾斜量を別入力する方式を候補として検討</x:v>
+      </x:c>
+      <x:c r="F16" s="12" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="G16" s="12" t="str">
+        <x:v>入力UI/軌道計算実装前</x:v>
+      </x:c>
+      <x:c r="H16" s="12" t="str">
+        <x:v>AimPoint関連特許に時計文字盤による方向表現の記載があるため重点確認</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="58" customHeight="1">
+      <x:c r="A17" s="12" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B17" s="12" t="str">
+        <x:v>傾斜・距離・速度から狙い/ブレーク算出</x:v>
+      </x:c>
+      <x:c r="C17" s="12" t="str">
+        <x:v>将来計画</x:v>
+      </x:c>
+      <x:c r="D17" s="12" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E17" s="12" t="str">
+        <x:v>局所傾斜とボール状態から軌道を計算し、将来的に狙い方向・必要速度等へ展開することを検討</x:v>
+      </x:c>
+      <x:c r="F17" s="12" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="G17" s="12" t="str">
+        <x:v>算出ロジック実装前</x:v>
+      </x:c>
+      <x:c r="H17" s="12" t="str">
+        <x:v>非侵害判断は未実施。関連特許ファミリー・対象国・有効請求項を実装前に確認</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F14">
     <x:cfRule type="expression" dxfId="2" priority="1">
@@ -1268,7 +1397,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16de4f9944ab415f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6df44b23f954f4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1391,6 +1520,58 @@
         <x:v>https://patents.justia.com/patent/11135498</x:v>
       </x:c>
     </x:row>
+    <x:row r="5" ht="95" customHeight="1">
+      <x:c r="A5" s="12" t="str">
+        <x:v>最優先</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>AimPoint関連 / Mark Sweeney</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>US 7,988,572 B1 / US 8,162,779 B1</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="str">
+        <x:v>Putting guide method and apparatus。距離、グリーンスピード、傾斜方向に対する角度等に応じ、開始速度・break量・aim point等を扱う。下り方向を基準とした角度を度数または時計文字盤で表す記載がある。Google Patentsでは両米国特許がExpired - Fee Related表示。</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="str">
+        <x:v>PuttPhysicsが検討する時計文字盤＋傾斜量入力、傾斜・距離・速度を用いた狙い/軌道計算と接点が大きい。局所傾斜を逐次適用する方式との差異を請求項単位で確認する必要。</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="str">
+        <x:v>独立請求項を構成要件分解。US7988572B1→US8162779B1の関係、関連出願、対象国、法的状態を確認。PuttPhysicsの具体実装案とクレームチャート化。</x:v>
+      </x:c>
+      <x:c r="G5" s="12" t="str">
+        <x:v>未判定</x:v>
+      </x:c>
+      <x:c r="H5" s="12" t="str">
+        <x:v>https://patents.google.com/patent/US8162779B1/en</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="95" customHeight="1">
+      <x:c r="A6" s="12" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>AimPoint関連 / Continuation-in-Part</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="str">
+        <x:v>US 2013/0116067 A1</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="str">
+        <x:v>Putting guide method and apparatus。straight-aimed puttからの距離、平均傾斜、距離等を用いた表形式/関係データからexpected breakを求める構成を含む公開。Google PatentsではAbandoned表示。</x:v>
+      </x:c>
+      <x:c r="E6" s="12" t="str">
+        <x:v>PuttPhysicsの将来の傾斜・ライン支援と機能目的が近い。一方、局所傾斜の時系列/空間逐次計算とは方式差がある可能性。</x:v>
+      </x:c>
+      <x:c r="F6" s="12" t="str">
+        <x:v>独立請求項13等のcomputer implemented methodを中心に、平均傾斜＋距離＋tabular/relational dataの要件とPuttPhysics案を比較。親・兄弟特許との重複も確認。</x:v>
+      </x:c>
+      <x:c r="G6" s="12" t="str">
+        <x:v>未判定</x:v>
+      </x:c>
+      <x:c r="H6" s="12" t="str">
+        <x:v>https://patents.google.com/patent/US20130116067A1/en</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="G2:G4">
@@ -1399,7 +1580,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41e09f78e78b47aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71bc6b9f6c714690"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1413,10 +1594,10 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="37" t="str">
+      <x:c r="A1" s="50" t="str">
         <x:v>PuttPhysics 競合・特許チェック表 Ver.1（プロトタイプ）</x:v>
       </x:c>
-      <x:c r="B1" t="str"/>
+      <x:c r="B1" s="12" t="str"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="48" t="str">
@@ -1472,6 +1653,14 @@
       </x:c>
       <x:c r="B8" s="12" t="str">
         <x:v>2026-08-16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="52" customHeight="1">
+      <x:c r="A9" s="12" t="str">
+        <x:v>2026-08-17 更新</x:v>
+      </x:c>
+      <x:c r="B9" s="12" t="str">
+        <x:v>局所傾斜・スネークライン共通モデル、時計文字盤＋傾斜量入力、AimPoint関連（US7988572B1 / US8162779B1 / US20130116067A1）を重点調査項目として追加。非侵害判断は未実施。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>